<commit_message>
Merge hero power selection into My Deck
Remove the standalone title control and show the selected power above the deck list. Choose unlocked powers in a compact integrated picker with keyboard focus handling and immediate persistence. Verify unlock gating, deck preservation, reload and new-duel application; update obsolete menu checks and the canonical rules workbook.
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Ra05350dfdec84dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rfa2cc636fc694db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R6db6af589ee54aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R570376a03dac4569"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R83489b63cf7b49b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rc3de1913e7514658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R1290c1c90f244bad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R548c6d1efb7c448c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc6553008a5b48df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddba218fc00a4de1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ac283f91884d9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7099095e79a47f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8488,7 +8488,7 @@
     </x:row>
     <x:row r="5" ht="67" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>Hero Powers are selected from the title-screen Hero Powers menu. Each first clear of chapters 1–10 unlocks the next player power permanently, in the order shown in that menu. Campaign bosses use fixed powers. Free-play opponents receive one random power from all ten. A selected Hero Power costs 2 mana and can be used once during its controller's turn.</x:v>
+        <x:v>Hero Powers are selected inside My Deck, above the current deck list. Each first clear of chapters 1–10 unlocks the next player power permanently, in the order shown in that menu. Campaign bosses use fixed powers. Free-play opponents receive one random power from all ten. A selected Hero Power costs 2 mana and can be used once during its controller's turn.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Update campaign reward ownership and Rick card name
Rick Prime renamed to Rick Clone (c045): renamed Rick Prime to Rick Clone
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R83489b63cf7b49b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rc3de1913e7514658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R1290c1c90f244bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R548c6d1efb7c448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R7e73e5b9d18a4ce7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R95fceb6e209841b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R8d8a8f945b054b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rc3b929e7df254928"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -779,7 +779,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Rick Prime</x:v>
+        <x:v>Rick Clone</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
         <x:f>D8&amp;"/"&amp;E8</x:f>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddba218fc00a4de1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eb8ff280d244ce1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7099095e79a47f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0678697af364830"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Move campaign filler rewards and rename Goku card
Mastered Ultra Instinct Goku renamed to Goku (c044): renamed Mastered Ultra Instinct Goku to Goku
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R7e73e5b9d18a4ce7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R95fceb6e209841b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R8d8a8f945b054b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rc3b929e7df254928"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rdb991a26780b4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Re04506672b674d55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rbeb5f620c9c74440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R7c53263595c24e49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -740,7 +740,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
-        <x:v>Mastered Ultra Instinct Goku</x:v>
+        <x:v>Goku</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
         <x:f>D7&amp;"/"&amp;E7</x:f>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eb8ff280d244ce1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc93a341741a543a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0678697af364830"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92bbc076bc004b59"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Fix boss gameplay controls and balance
Sonic stats changed (c085): changed Sonic ATK from 6 to 5

Planetary Defense Grid (c177): corrected effect text to friendly Taunt minions
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rdb991a26780b4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Re04506672b674d55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rbeb5f620c9c74440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R7c53263595c24e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R156bb51a3bb04b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R501caadecfc141d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R62f6c7cedc834c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R27eb656372814c27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2634,7 +2634,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I55" s="18" t="str">
-        <x:v>Taunt. Passive: All other Taunt minions have +2/+2</x:v>
+        <x:v>Taunt. Passive: All other friendly Taunt minions have +2/+2</x:v>
       </x:c>
       <x:c r="J55" s="18" t="str">
         <x:v>The shield watches from orbit.</x:v>
@@ -3279,10 +3279,10 @@
       </x:c>
       <x:c r="C72" s="23" t="str">
         <x:f>D72&amp;"/"&amp;E72</x:f>
-        <x:v>6/3</x:v>
+        <x:v>5/3</x:v>
       </x:c>
       <x:c r="D72" s="21" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E72" s="21" t="n">
         <x:v>3</x:v>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc93a341741a543a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb587e59fac644c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92bbc076bc004b59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea53c4193a044d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh card workbook snapshot
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R156bb51a3bb04b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R501caadecfc141d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R62f6c7cedc834c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R27eb656372814c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R72179be287494d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R27da00817f26489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R55086e4aff6f4ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R47a1453d82ab4a69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb587e59fac644c0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcac9b921c0ff4c37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea53c4193a044d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b35a0324bad4c1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8486,9 +8486,9 @@
         <x:v>Each player draws from their own shuffled thirty-card deck and opens with 3 cards. In solo and campaign play, Player One may replace any number once during the mulligan. In hotseat, both players may replace cards once, privately and in order. The second player also receives The Coin.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="67" customHeight="1">
+    <x:row r="5" ht="84" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>Hero Powers are selected inside My Deck, above the current deck list. Each first clear of chapters 1–10 unlocks the next player power permanently, in the order shown in that menu. Campaign bosses use fixed powers. Free-play opponents receive one random power from all ten. A selected Hero Power costs 2 mana and can be used once during its controller's turn.</x:v>
+        <x:v>Hero Powers are selected inside My Deck, above the current deck list. Each first clear of the first ten universes unlocks the next player power permanently, in the order shown in that menu. Collection bosses use fixed powers. Free-play opponents receive one random player power from all ten. A selected Hero Power costs 2 mana and can be used once during its controller's turn.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Refine boss powers and duel presentation
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R72179be287494d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R27da00817f26489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R55086e4aff6f4ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R47a1453d82ab4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R43691d1a4bd74495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R33d9218ce8984b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rf3cb9d15b9c04909"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R4e756f9d1aeb4934"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7736,7 +7736,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcac9b921c0ff4c37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5016662cc9cf4da3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8456,7 +8456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b35a0324bad4c1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59207d1b26514a84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8478,12 +8478,12 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>Both cores begin at 75 health. Reduce the opposing core to zero to win.</x:v>
+        <x:v>Both cores begin at 50 health. Reduce the opposing core to zero to win.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="67" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>Each player draws from their own shuffled thirty-card deck and opens with 3 cards. In solo and campaign play, Player One may replace any number once during the mulligan. In hotseat, both players may replace cards once, privately and in order. The second player also receives The Coin.</x:v>
+        <x:v>Each player draws from their own shuffled thirty-card deck and opens with 3 cards. In solo and campaign play, Player One may replace any number once during the mulligan. In hotseat, both players may replace cards once, privately and in order. The second hotseat player also receives The Coin.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="84" customHeight="1">

</xml_diff>

<commit_message>
Unfreeze lore ranking sheet
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R0d549da917aa41db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R30acf3f7e15e4455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rbdedd6f0eaf64e6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R3f24e8fb0e554023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R5fc0b2abe3a24b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R1e78db5038ff4161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rc3071fba0e33456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R9fda9a7b1efd441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rf5840bbc6f454678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="Rb60ce86f6e224f9e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7839,7 +7839,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d6d9386966f43f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb96f4168fc54b9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8559,7 +8559,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29104f42ce794b46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8182944af5bf4582"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18119,7 +18119,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0894a1f916254f55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c39d4ca1694ed3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add lore ranking rules tab
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R1e78db5038ff4161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rc3071fba0e33456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R9fda9a7b1efd441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rf5840bbc6f454678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="Rb60ce86f6e224f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R87b3367f336341cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rf27afb44528e4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R106dd62e0d264102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R75817b6e7c4144e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R267bf04e025d4774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R4d4affb271ea43a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +68,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +105,11 @@
         <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -111,7 +117,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -218,6 +224,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -7839,7 +7866,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb96f4168fc54b9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f5d81100c04462c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8559,7 +8586,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8182944af5bf4582"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R740211b80f52475f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18119,7 +18146,245 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c39d4ca1694ed3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c718354f99141b6"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="122" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="37" t="str">
+        <x:v>Lore Ranking Rules</x:v>
+      </x:c>
+      <x:c r="B1" s="37"/>
+      <x:c r="C1" s="37"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="9"/>
+      <x:c r="B2" s="9"/>
+      <x:c r="C2" s="9"/>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="40" t="str">
+        <x:v>#</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="50" customHeight="1">
+      <x:c r="A4" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="42" t="str">
+        <x:v>Screen-oriented canon</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="str">
+        <x:v>Use the screen version when one exists. Anime, film, or TV portrayals take priority over manga, comic, novel, or other source-material versions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="50" customHeight="1">
+      <x:c r="A5" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="42" t="str">
+        <x:v>Prime condition</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>Rank characters in their strongest normally accessible canonical condition, not while weakened by illness, age, injury, or an explicitly diminished state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="50" customHeight="1">
+      <x:c r="A6" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="42" t="str">
+        <x:v>Ignore world-entry restrictions</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>Do not count restrictions that only govern summoning, entry, or initial manifestation in the battlefield/world. Once present, evaluate the character without those entry-only restrictions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="50" customHeight="1">
+      <x:c r="A7" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="42" t="str">
+        <x:v>Standardized supernatural systems</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>Treat magic, mana, chakra, nen, ki, cursed energy, and analogous supernatural energy systems as mutually interactive for cross-setting comparisons.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="50" customHeight="1">
+      <x:c r="A8" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="42" t="str">
+        <x:v>Interoperability is not equalization</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>Standardization lets different power systems interact; it does not make their reserves, efficiency, mechanics, or potency equal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="67" customHeight="1">
+      <x:c r="A9" s="41" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="42" t="str">
+        <x:v>Temporary peak forms</x:v>
+      </x:c>
+      <x:c r="C9" s="43" t="str">
+        <x:v>Include transformations or peak states the character can access through their own normal abilities, even if time-limited. Exclude one-off external empowerment, borrowed power, possession, or special plot-only amps unless that version is explicitly the listed entry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="42" t="str">
+        <x:v>No continuity composites</x:v>
+      </x:c>
+      <x:c r="C10" s="43" t="str">
+        <x:v>Do not combine unrelated adaptations or continuities. Use the version implied by the Origin and Version fields.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
+      <x:c r="A11" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="42" t="str">
+        <x:v>Screen feats stay screen feats</x:v>
+      </x:c>
+      <x:c r="C11" s="43" t="str">
+        <x:v>Source material may clarify terminology or mechanics when useful, but manga/comic/novel-only feats should not be imported into a screen-oriented version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="67" customHeight="1">
+      <x:c r="A12" s="41" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="42" t="str">
+        <x:v>Evidence priority</x:v>
+      </x:c>
+      <x:c r="C12" s="43" t="str">
+        <x:v>Demonstrated canonical feats carry the most weight. Clear narrator, creator, or in-universe statements can supplement them. Hyperbole, jokes, promotional claims, and vague 'infinite power' language should not automatically be treated literally.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
+      <x:c r="A13" s="41" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="42" t="str">
+        <x:v>Scaling</x:v>
+      </x:c>
+      <x:c r="C13" s="43" t="str">
+        <x:v>Direct and consistent scaling from other characters is allowed. Record defensible comparisons in the Scaling field, but avoid long speculative chains or one-off outlier scaling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="50" customHeight="1">
+      <x:c r="A14" s="41" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="42" t="str">
+        <x:v>Equipment and summons</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>Standard equipment, permanently owned gear, and summons that are part of the character's normal kit count. Temporary borrowed gear and unrelated allies do not.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="50" customHeight="1">
+      <x:c r="A15" s="41" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="str">
+        <x:v>Groups and objects</x:v>
+      </x:c>
+      <x:c r="C15" s="43" t="str">
+        <x:v>Evaluate groups, armies, vehicles, artifacts, and structures as the exact listed entity rather than forcing them into individual-character assumptions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="50" customHeight="1">
+      <x:c r="A16" s="41" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="42" t="str">
+        <x:v>Combat limitations still count</x:v>
+      </x:c>
+      <x:c r="C16" s="43" t="str">
+        <x:v>Keep limitations that affect actual combat performance, such as cooldowns, stamina, range, concentration, activation conditions, ammunition, required gestures, or exploitable weaknesses.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="50" customHeight="1">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="42" t="str">
+        <x:v>Quantity is numeric only</x:v>
+      </x:c>
+      <x:c r="C17" s="43" t="str">
+        <x:v>Use only a number in Quantity. Use 1 for a single character/entity unless the listed entry explicitly represents multiple members; for groups, use the exact listed count when known.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="50" customHeight="1">
+      <x:c r="A18" s="41" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="42" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="C18" s="43" t="str">
+        <x:v>Prefer specific canonical references where practical, such as season/episode, film, chapter, or issue. Reliable secondary sources may be added for verification or terminology, but should not replace primary canon evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="84" customHeight="1">
+      <x:c r="A19" s="41" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="42" t="str">
+        <x:v>House Rules</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="str">
+        <x:v>Custom deviations override normal canon where explicitly stated on a card. Neo and Morpheus: treat their Matrix-enhanced abilities as functioning in the real world as well; they perceive reality as Matrix-like code and retain their Matrix superhuman abilities outside the simulation. Light Yagami: Ryuk actively assists Light when useful, including using his Shinigami Eyes to identify a target's true name for Light.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="84" customHeight="1">
+      <x:c r="A20" s="41" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="42" t="str">
+        <x:v>Source-material peek</x:v>
+      </x:c>
+      <x:c r="C20" s="43" t="str">
+        <x:v>When a screen version does not yet provide enough information to judge a character's intended power level, later manga/comic/source-material feats may be consulted as a limited 'peek' to understand the likely power bracket, toolkit, or scaling. Peek material must be clearly labeled in Scaling or Sources and should not be silently imported as an on-screen feat. Screen-demonstrated feats remain the primary evidence whenever available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="101" customHeight="1">
+      <x:c r="A21" s="41" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="42" t="str">
+        <x:v>Demonstrated power utilization</x:v>
+      </x:c>
+      <x:c r="C21" s="43" t="str">
+        <x:v>Rank practical lore threat, not only a power's theoretical ceiling. How reliably, intelligently and creatively an entity converts its abilities, equipment or hax into actual results matters. Proven planning, consistency and successful exploitation of narrow powers can raise effective threat; repeated self-sabotage, design flaws, poor judgment, failure to capitalize, or a long canon pattern of failing to secure wins despite powerful tools can lower it. Do not overreact to one isolated plot loss, but repeated demonstrated performance is valid evidence.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Polish duel board and boss mechanics
Card changes:\n- Sandworm (c006): effect id small_attack_ward_3 to small_attack_ward_2, text\n- Ragnaros (c031): health 4 to 3\n- Godzilla (c076): text\n- Tech Hub (c141): keywords Divine Shield to Divine Shield;Passive, timing ongoing to passive, text
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R87b3367f336341cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rf27afb44528e4864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R106dd62e0d264102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R75817b6e7c4144e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R267bf04e025d4774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R4d4affb271ea43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R181b8fd6e27349e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R23e630403d044eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R2219b462f3a94421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rba9d0ff238114c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R2adc1ee602854140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R04da4175e12b4960"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2503,7 +2503,7 @@
         <x:v>c072</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="42" customHeight="1">
+    <x:row r="49" ht="44" customHeight="1">
       <x:c r="A49" s="22" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -2530,7 +2530,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I49" s="18" t="str">
-        <x:v>Passive: Deal 2 damage to all enemies each time you take damage</x:v>
+        <x:v>Passive: Deal 2 damage to all enemy minions each time you take damage</x:v>
       </x:c>
       <x:c r="J49" s="18" t="str">
         <x:v>Laser breathing</x:v>
@@ -5398,13 +5398,13 @@
       </x:c>
       <x:c r="C123" s="24" t="str">
         <x:f>D123&amp;"/"&amp;E123</x:f>
-        <x:v>4/4</x:v>
+        <x:v>4/3</x:v>
       </x:c>
       <x:c r="D123" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E123" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F123" s="24" t="str">
         <x:v>Rare</x:v>
@@ -5494,7 +5494,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I125" s="18" t="str">
-        <x:v>Taunt. Passive: Cannot be damaged by minions with 3 or less ATK</x:v>
+        <x:v>Taunt. Passive: Cannot be damaged by minions with 2 or less ATK</x:v>
       </x:c>
       <x:c r="J125" s="18" t="str">
         <x:v>The desert itself has teeth.</x:v>
@@ -6508,7 +6508,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I151" s="18" t="str">
-        <x:v>Divine Shield. Ongoing: Give all other friendly Tech minions +2/+1</x:v>
+        <x:v>Divine Shield. Passive: Give all other friendly Tech minions +2/+1</x:v>
       </x:c>
       <x:c r="J151" s="18" t="str">
         <x:v>Every machine came from somewhere. This is that somewhere</x:v>
@@ -7866,7 +7866,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f5d81100c04462c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55d07fd55e954dbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8586,7 +8586,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R740211b80f52475f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb3cbac205c543d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8633,7 +8633,7 @@
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="str">
-        <x:v>Play a hand card into one of five board slots by paying its cost. Effects that summon minions also need an open slot.</x:v>
+        <x:v>Play a hand card into one of four board slots by paying its cost. Effects that summon minions also need an open slot.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="50" customHeight="1">
@@ -18146,7 +18146,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c718354f99141b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R868e63ea1492468b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Make critical health warnings visible
Card changes:\n- Ragnaros (c031): attack 4 to 3, health remains 3
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R181b8fd6e27349e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R23e630403d044eed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R2219b462f3a94421"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rba9d0ff238114c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R2adc1ee602854140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R04da4175e12b4960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R2a8f48e0843c485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R43a5d9f9643c47ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rbd1dbe47f26e42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rb706e65f37d445ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R4bea50bcf82a46ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="Rf86945cb35e84375"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5398,10 +5398,10 @@
       </x:c>
       <x:c r="C123" s="24" t="str">
         <x:f>D123&amp;"/"&amp;E123</x:f>
-        <x:v>4/3</x:v>
+        <x:v>3/3</x:v>
       </x:c>
       <x:c r="D123" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E123" s="22" t="n">
         <x:v>3</x:v>
@@ -7866,7 +7866,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55d07fd55e954dbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R208a816aee9d412b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8586,7 +8586,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb3cbac205c543d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30332dcb230b4267"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18146,7 +18146,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R868e63ea1492468b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31aaac2c4e394dff"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Rebuild mobile play and clean public documentation
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R8eba4a9a0b874e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rf72bc3291f544030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R29045237e1fb4733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R41f2a3c94ab444ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R995bfb206deb46a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="Rd41c74f213084f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R71f6272aa2b244dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rf6faee656cbf442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R2aa24c62f52b47ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rd0ab9970a1f64a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R04b4955f7ac54480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R3669a3c922b843e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7827,7 +7827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cc4aee803946ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf6e755b6bc94c00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8547,7 +8547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08cf3cf2640547c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a2f2ca122564361"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8572,64 +8572,69 @@
         <x:v>Both cores begin at 50 health. Reduce the opposing core to zero to win.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="67" customHeight="1">
+    <x:row r="4" ht="50" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>Each player draws from their own shuffled thirty-card deck and opens with 3 cards. In solo and campaign play, Player One may replace any number once during the mulligan. In hotseat, both players may replace cards once, privately and in order. The second hotseat player also receives The Coin.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="84" customHeight="1">
+        <x:v>Each player draws from their own shuffled 30-card deck and opens with 3 cards. Solo play offers one opening mulligan; hotseat offers one private mulligan per player. The second hotseat player receives The Coin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>Hero Powers are selected inside My Deck, above the current deck list. Each first clear of the first ten universes unlocks the next player power permanently, in the order shown in that menu. Collection bosses use fixed powers. Free-play opponents receive one random player power from all ten. A selected Hero Power costs 2 mana and can be used once during its controller's turn.</x:v>
+        <x:v>At the start of a turn, draw one card. Mana begins at 1, refills each turn, and increases by one up to 10.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>At the start of a turn, draw one card. Mana starts at 1, refills each turn, and increases by one each turn up to 10.</x:v>
+        <x:v>Your hand holds at most 10 cards. A card drawn into a full hand burns.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="9" t="str">
-        <x:v>Your hand holds at most 10 cards. A card drawn into a full hand burns and is discarded.</x:v>
+        <x:v>Pay a card's mana cost to play it. Each player has four board slots. Summons need an available slot.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="str">
-        <x:v>Play a hand card into one of four board slots by paying its cost. Effects that summon minions also need an open slot.</x:v>
+        <x:v>A newly played minion normally sleeps until its owner's next turn. Charge allows an immediate attack.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="50" customHeight="1">
       <x:c r="A9" s="9" t="str">
-        <x:v>A minion is asleep for the turn it enters play and normally waits until its owner's next turn before attacking. A Chained minion is unavailable for its first two owner turns and cannot be targeted by attacks or effects while chained.</x:v>
+        <x:v>A ready minion attacks once per turn. Combat damage is simultaneous: defenders hit back even when the attack destroys them.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="str">
-        <x:v>A minion can attack once per turn. A minion with 0 ATK can still attack, but deals no damage.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+        <x:v>Taunt prevents attacks on the opposing core until its defence is removed, unless an effect explicitly bypasses it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
       <x:c r="A11" s="9" t="str">
-        <x:v>Combat is simultaneous: attacker and defender deal damage to each other, even when the attack kills the defender.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="50" customHeight="1">
+        <x:v>Chained minions lose two of their own turns. They cannot attack, activate Passive or Ongoing effects, or be targeted while chained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="9" t="str">
-        <x:v>Taunt must be dealt with before attacks can reach the opposing core, unless an effect or relic explicitly bypasses that defence.</x:v>
+        <x:v>Freeze costs one attack turn. A frozen minion remains targetable and keeps its Passive effects.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="50" customHeight="1">
       <x:c r="A13" s="9" t="str">
-        <x:v>Silence strips printed text, keywords, and stat buffs at once. A minion pumped above its printed stats falls back to them; a minion pushed below them stays there. A silenced minion's Divine Shield blocks nothing while the silence holds.</x:v>
+        <x:v>Silence disables printed abilities and keywords, removes positive stat buffs, and retains stat reductions. It never heals a damaged minion.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="50" customHeight="1">
       <x:c r="A14" s="9" t="str">
-        <x:v>When a player's own deck and bottom-deck cards are empty, drawing causes escalating fatigue damage: 1, then 2, then 3, and so on.</x:v>
+        <x:v>Each minion can carry up to two relics. Returning it to hand discards its attached relics; its death destroys them unless their text says otherwise.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="50" customHeight="1">
       <x:c r="A15" s="9" t="str">
-        <x:v>Nothing damages a core automatically just because a turn starts; core damage comes from a minion attacking it or from an effect that explicitly says it damages a core.</x:v>
+        <x:v>Earned player Hero Powers cost 2 mana and can be used once per turn. Boss powers have their own printed costs or passive rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="9" t="str">
+        <x:v>When your own draw pile and bottom pile are empty, attempts to draw cause escalating fatigue damage: 1, 2, 3, and so on.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18106,7 +18111,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda33bc79b39c4438"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc904b592c92d4b99"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add first-victory comic and polish title, Discover, phone layout and Batman
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R71f6272aa2b244dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="Rf6faee656cbf442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R2aa24c62f52b47ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rd0ab9970a1f64a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R04b4955f7ac54480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R3669a3c922b843e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R1c14f5f7ac5c41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R50e1762d124e461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R2c7f850bff594b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R9ae9ce24613b4f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R09e75aef9c354379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R7496df26eb48424c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6577,7 +6577,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F153" s="24" t="str">
-        <x:v>Epic</x:v>
+        <x:v>Mythic</x:v>
       </x:c>
       <x:c r="G153" s="24" t="str">
         <x:v>Tech</x:v>
@@ -6586,7 +6586,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I153" s="18" t="str">
-        <x:v>Battlecry: Choose an enemy minion. Choose one gadget: Freeze it; Silence it; or give it -3 ATK</x:v>
+        <x:v>Battlecry: Choose an enemy minion. Choose one gadget: Freeze it; Silence it; or give it -2 ATK</x:v>
       </x:c>
       <x:c r="J153" s="18" t="str">
         <x:v>Preparation beats power.</x:v>
@@ -7827,7 +7827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf6e755b6bc94c00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51ed1c1e6b7e4b45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8547,7 +8547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a2f2ca122564361"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra742e37bf91e46eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8670,7 +8670,7 @@
       </x:c>
       <x:c r="B2" s="8" t="n">
         <x:f>COUNTIF(Cards!F2:F184,A2)</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="8" t="n">
@@ -8704,7 +8704,7 @@
       </x:c>
       <x:c r="B4" s="8" t="n">
         <x:f>COUNTIF(Cards!F2:F184,A4)</x:f>
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="8" t="n">
@@ -18111,7 +18111,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc904b592c92d4b99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68553e0ee1324ebc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Polish gallery and consolidate Gums and Nyan artwork; use 30 HP cores
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rd467d90e666c4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R81a6300fe6b8428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R4c770d000c644efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R36ff3a8a866d4842"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R2543f7f8db7b481a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R785aeb3523e44c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rb6dad1b5d9ee4daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R6de9d8e762424a97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R12fdff001a9e46d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rbb251028ad744570"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R0e3fa6a6f0944358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="Rb042457277c24aa0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7827,7 +7827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R046ef93b42344ae4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0c43b9cea14ae6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8547,7 +8547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b4bc0785ca746fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d21e6a9bcb4b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8569,7 +8569,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>Both cores begin at 50 health. Reduce the opposing core to zero to win.</x:v>
+        <x:v>Both cores begin at 30 health. Reduce the opposing core to zero to win.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="50" customHeight="1">
@@ -18111,7 +18111,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e06771481424c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60f240e6d639456a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Revise Doom Slayer, Meteor, Carrier Strike Group, Guts, RoboCop, An Order of Heavy Knights and Nine Hashira
Apply requested stats and passives. Replace Nine Hashira forced attacks with a Good-minion-scaled enemy volley. Add Rebirth, Bearer and Evades tooltips and adjust Stand Arrow and Walter White framing.
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rb6dad1b5d9ee4daa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R6de9d8e762424a97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R12fdff001a9e46d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rbb251028ad744570"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R0e3fa6a6f0944358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="Rb042457277c24aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R9d44e9455d50439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R1a1a37d465874c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R54f67372c5c24ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R14c89e81505743c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="Rd68ddc203a1541e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R8352d06fbdeb4a94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1576,10 +1576,10 @@
       </x:c>
       <x:c r="C25" s="24" t="str">
         <x:f>D25&amp;"/"&amp;E25</x:f>
-        <x:v>3/8</x:v>
+        <x:v>4/8</x:v>
       </x:c>
       <x:c r="D25" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E25" s="22" t="n">
         <x:v>8</x:v>
@@ -1594,7 +1594,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I25" s="18" t="str">
-        <x:v>Passive: Deal triple damage to Evil minions. Whenever Doom Slayer kills an Evil minion, heal him for 3 HP</x:v>
+        <x:v>Passive: Deal double damage to Evil minions. Whenever Doom Slayer kills an Evil minion, heal him for 3 HP</x:v>
       </x:c>
       <x:c r="J25" s="18" t="str">
         <x:v>He cleaned Hell and came back.</x:v>
@@ -1888,13 +1888,13 @@
       </x:c>
       <x:c r="C33" s="24" t="str">
         <x:f>D33&amp;"/"&amp;E33</x:f>
-        <x:v>4/3</x:v>
+        <x:v>4/4</x:v>
       </x:c>
       <x:c r="D33" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E33" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F33" s="24" t="str">
         <x:v>Rare</x:v>
@@ -3643,10 +3643,10 @@
       </x:c>
       <x:c r="C78" s="23" t="str">
         <x:f>D78&amp;"/"&amp;E78</x:f>
-        <x:v>1/5</x:v>
+        <x:v>2/5</x:v>
       </x:c>
       <x:c r="D78" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="21" t="n">
         <x:v>5</x:v>
@@ -5221,7 +5221,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I118" s="13" t="str">
-        <x:v>Battlecry: Choose an enemy Evil minion. Every friendly minion attacks it immediately</x:v>
+        <x:v>Battlecry: Deal 1 damage to all enemy minions for each friendly Good minion</x:v>
       </x:c>
       <x:c r="J118" s="13" t="str">
         <x:v>Nine pillars holding the sky</x:v>
@@ -6079,7 +6079,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I140" s="13" t="str">
-        <x:v>Passive: Gains +2/+2 for each 20 HP your Core is missing</x:v>
+        <x:v>Passive: Gains +1/+1 for each 5 HP your Core is missing</x:v>
       </x:c>
       <x:c r="J140" s="13" t="str">
         <x:v>Struggle is the only answer.</x:v>
@@ -6391,7 +6391,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I148" s="13" t="str">
-        <x:v>Passive: Deal 3x damage against Evil minions</x:v>
+        <x:v>Passive: Deal double damage against Evil minions</x:v>
       </x:c>
       <x:c r="J148" s="13" t="str">
         <x:v>Uphold the law</x:v>
@@ -7105,7 +7105,7 @@
         <x:v>c143</x:v>
       </x:c>
     </x:row>
-    <x:row r="167" ht="42" customHeight="1">
+    <x:row r="167" ht="44" customHeight="1">
       <x:c r="A167" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -7132,7 +7132,7 @@
         <x:v>Neutral</x:v>
       </x:c>
       <x:c r="I167" s="18" t="str">
-        <x:v>Passive: While you control a Taunt minion, this has +1/+1</x:v>
+        <x:v>Passive: Gain +1/+1 for every friendly Taunt or Divine Shield minion</x:v>
       </x:c>
       <x:c r="J167" s="18" t="str">
         <x:v>Honor. Duty</x:v>
@@ -7827,7 +7827,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0c43b9cea14ae6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd3f19608dd64a90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8547,7 +8547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d21e6a9bcb4b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34175c67ec8743ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18111,7 +18111,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60f240e6d639456a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57a84f33d0254869"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Local Duel and Arena names, opening lore book, deck rename and delete, card buffs
- Title: "2 players" becomes Local Duel, Rift Draft becomes Arena.
- The Lore button is a 3D book whose cover opens on hover onto a lit page.
- Decks can be renamed and deleted; the Starter Deck stays protected.
  Choose Hero Power moves to the top of the deck list in its own teal.
- Gyoro Gyoro 2/6, Pillar Men 5/4, Frieren 6 HP and every relic cast.
- Grand Master Oogway (c094): text; rescues every ally, never Chained.
- Pandora's Box now gives its bearer the effect of a random other relic.
- The boss runner saves quick or partial runs to their own file.
- Release rebuilt into play/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materials/Convergence card stat excel sheet.xlsx
+++ b/materials/Convergence card stat excel sheet.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R28c27377e00f4fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R82527bd88ddd4841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rd1a68b2c35e74501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R1c2d682a665c4af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="Rb9e87306b7fe46c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="Rf4a7efd15f7f49d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Re3d09661d95247b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relics" sheetId="2" r:id="R75b3dc41fad242c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Ree7d6bcd11964017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Re309b9d298a7414d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking" sheetId="5" r:id="R4e17c67c500b4dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Ranking Rules" sheetId="6" r:id="R55814f50e8ae4351"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -112,7 +112,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3088,7 +3094,7 @@
         <x:v>c087</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="44" customHeight="1">
+    <x:row r="64" ht="42" customHeight="1">
       <x:c r="A64" s="21" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -3097,13 +3103,13 @@
       </x:c>
       <x:c r="C64" s="23" t="str">
         <x:f>D64&amp;"/"&amp;E64</x:f>
-        <x:v>2/5</x:v>
+        <x:v>2/6</x:v>
       </x:c>
       <x:c r="D64" s="21" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E64" s="21" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F64" s="23" t="str">
         <x:v>Legendary</x:v>
@@ -3115,7 +3121,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I64" s="13" t="str">
-        <x:v>Passive: The first time you cast a relic each turn, discover another relic</x:v>
+        <x:v>Passive: Whenever you cast a relic, discover another relic</x:v>
       </x:c>
       <x:c r="J64" s="13" t="str">
         <x:v>Every spell is worth remembering.</x:v>
@@ -3973,7 +3979,7 @@
         <x:v>Good</x:v>
       </x:c>
       <x:c r="I86" s="13" t="str">
-        <x:v>Divine Shield. Passive: Once per turn, when another friendly minion would die, return it to your hand instead and Chain Oogway</x:v>
+        <x:v>Divine Shield. Passive: When another friendly minion would die, return it to your hand instead</x:v>
       </x:c>
       <x:c r="J86" s="13" t="str">
         <x:v>Patience</x:v>
@@ -4891,13 +4897,13 @@
       </x:c>
       <x:c r="C110" s="23" t="str">
         <x:f>D110&amp;"/"&amp;E110</x:f>
-        <x:v>1/4</x:v>
+        <x:v>2/6</x:v>
       </x:c>
       <x:c r="D110" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E110" s="21" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F110" s="23" t="str">
         <x:v>Epic</x:v>
@@ -5281,10 +5287,10 @@
       </x:c>
       <x:c r="C120" s="23" t="str">
         <x:f>D120&amp;"/"&amp;E120</x:f>
-        <x:v>4/4</x:v>
+        <x:v>5/4</x:v>
       </x:c>
       <x:c r="D120" s="21" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E120" s="21" t="n">
         <x:v>4</x:v>
@@ -7827,7 +7833,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R880d0b4458324faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1dd7ffecd824c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8252,7 +8258,7 @@
         <x:v>Pandora's Box</x:v>
       </x:c>
       <x:c r="C21" s="18" t="str">
-        <x:v>The bearer gains +4/+4. It dies at the start of your next turn</x:v>
+        <x:v>The bearer gains an effect of a random relic</x:v>
       </x:c>
       <x:c r="D21" s="18" t="str">
         <x:v>RELIC</x:v>
@@ -8547,7 +8553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2842a1a2ede4f76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc154ec3e27f54fa3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8574,7 +8580,7 @@
     </x:row>
     <x:row r="4" ht="50" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>Each player draws from their own shuffled 30-card deck and opens with 3 cards. Solo play offers one opening mulligan; hotseat offers one private mulligan per player. The second hotseat player receives The Coin.</x:v>
+        <x:v>Each player draws from their own shuffled 30-card deck and opens with 3 cards. Solo play offers one opening mulligan; Local Duel offers one private mulligan per player. The second Local Duel player receives The Coin.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -18111,7 +18117,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7af84ab7b74485d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ac5f3e07c244c4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>